<commit_message>
NHANES code alc_qty and smk_qty 0.
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHANES11.xlsx
+++ b/baseline/data_processing_elements-NHANES11.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\NHANES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20E863DC-F665-4E61-88CC-40E4F7E23EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A153B386-4332-4473-9E30-1ED3AC4B2EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3161BE6F-2E10-4AFE-B2DF-B65F0CC4B714}"/>
   </bookViews>
@@ -2282,38 +2282,12 @@
 . = Missing</t>
   </si>
   <si>
-    <t>SMD650;
-SMD641</t>
-  </si>
-  <si>
-    <t>Avg # cigarettes/day during past 30 days;
-# days smoked cigs during past 30 days</t>
-  </si>
-  <si>
     <t>During the past 30 days, on the days that {you/SP} smoked, about how many cigarettes did {you/s/he} smoke per day?;
 On how many of the past 30 days did {you/SP} smoke a cigarette?</t>
   </si>
   <si>
     <t>Both males and females 12 YEARS - 150 YEARS
 1 PACK EQUALS 20 CIGARETTES. IF LESS THAN 1 PER DAY, ENTER 1. IF 95 OR MORE PER DAY, ENTER 95. ENTER NUMBER (OF CIGARETTES) (PER DAY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 to 80 = Range of Values
-1 = 1 cigarette or less
-95 = 95 cigarettes or more
-777 = Refused
-999 = Don't know
-. = Missing
-0 to 30 = Range of Values
-77 = Refused
-99 = Don't know
-. = Missing	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">case_when(
-SMD650 %in% c(1:95) &amp; SMD641 %in% c(0:30) ~ round(SMD650*SMD641/(30/7), 2);
-ELSE ~ NA_real_)
-</t>
   </si>
   <si>
     <t>How much sleep do you get (hours)?</t>
@@ -3135,15 +3109,6 @@
   </si>
   <si>
     <t>case_when(
-ALQ120Q %in% c(NA, 777, 999) | ALQ120U %in% c(NA, 7, 9) | ALQ130 %in%c(NA, 777, 999) ~ NA_real_;
-ALQ120Q == 0 ~ 0;
-ALQ120U == 1 ~ round( 14*ALQ130*ALQ120Q, 2);
-ALQ120U == 2 ~ round( 14*ALQ130*ALQ120Q*((12*7)/365.25), 2 );
-ALQ120U == 3 ~ round( 14*ALQ130*ALQ120Q * (7/365.25), 2);
-ELSE ~ NA_real_)</t>
-  </si>
-  <si>
-    <t>case_when(
 DR1_300 == 2 &amp; ! is.na(DR1TKCAL) &amp; DR1TKCAL &gt;0 ~ DR1TKCAL;
 DR2_300 == 2 &amp; ! is.na(DR2TKCAL) &amp; DR2TKCAL &gt;0 ~ DR2TKCAL;
 ELSE ~ NA_real_)</t>
@@ -3379,19 +3344,12 @@
     <t>Study-specific information is based on amount of food eaten yesterday, and only used if the participant responded that it was a usual amount. There are outlier values in the output.</t>
   </si>
   <si>
-    <t xml:space="preserve">The study-specific information was based on responses about alcohol use in the past 12 months. Mean grams of alcohol per standard drink in the United States (14g) was used for calculations. 
-</t>
-  </si>
-  <si>
     <t>1 year = 365.25 days
 https://iard.org/science-resources/detail/drinking-guidelines-general-population;
 If the participant had more than 95 drink at each sitting, values of 95 drinks and over were topcoded at 95. But this did not happen.</t>
   </si>
   <si>
     <t>Study participants were only considered as having smoked if they have smoked at least 100 cigarettes in their entire life.</t>
-  </si>
-  <si>
-    <t>The study-specific maximum was 95 cigarettes a day, and the minimum was  1 cigarette a day.</t>
   </si>
   <si>
     <t>The study-specific category "12 hours or more" was coded as 12.</t>
@@ -3623,6 +3581,55 @@
   </si>
   <si>
     <t>Didn't find this variable in this wave, but added comment about leisure activities.</t>
+  </si>
+  <si>
+    <t>SMQ020;
+SMD650;
+SMD641</t>
+  </si>
+  <si>
+    <t>Smoked at least 100 cigarettes in life;
+Avg # cigarettes/day during past 30 days;
+# days smoked cigs during past 30 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = Yes;
+2 = No;
+7 = Refused;
+9 = Don't know;
+. = Missing	
+2 to 80 = Range of Values
+1 = 1 cigarette or less
+95 = 95 cigarettes or more
+777 = Refused
+999 = Don't know
+. = Missing
+0 to 30 = Range of Values
+77 = Refused
+99 = Don't know
+. = Missing	</t>
+  </si>
+  <si>
+    <t>Non-smokers (never smoked at least 100 cigarettes in life) were coded as 0. The study-specific maximum for Avg # cigarettes/day during past 30 days was 95 cigarettes a day, and the minimum was  1 cigarette a day.</t>
+  </si>
+  <si>
+    <t>case_when(
+SMQ020 == 2 ~ 0L;
+SMD650 %in% c(1:95) &amp; SMD641 %in% c(0:30) ~ round(SMD650*SMD641/(30/7), 2);
+ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t>case_when(
+ALQ120Q == 0 ~ 0;
+ALQ120Q %in% c(NA, 777, 999) | ALQ130 %in%c(NA, 777, 999) ~ NA_real_;
+ALQ120U == 1 ~ round( 14*ALQ130*ALQ120Q, 2);
+ALQ120U == 2 ~ round( 14*ALQ130*ALQ120Q*((12*7)/365.25), 2 );
+ALQ120U == 3 ~ round( 14*ALQ130*ALQ120Q * (7/365.25), 2);
+ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-drinkers were coded as 0. The study-specific information was based on responses about alcohol use in the past 12 months. Mean grams of alcohol per standard drink in the United States (14g) was used for calculations. 
+</t>
   </si>
 </sst>
 </file>
@@ -4157,7 +4164,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>10</v>
@@ -4166,7 +4173,7 @@
         <v>11</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="O1" s="9" t="s">
         <v>12</v>
@@ -4187,10 +4194,10 @@
         <v>17</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="V1" s="10" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="W1" s="10" t="s">
         <v>18</v>
@@ -4305,7 +4312,7 @@
         <v>473</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="165" x14ac:dyDescent="0.25">
@@ -4343,7 +4350,7 @@
         <v>473</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
@@ -4384,7 +4391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -4413,7 +4420,7 @@
         <v>472</v>
       </c>
       <c r="U6" s="12" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="V6" s="3" t="s">
         <v>474</v>
@@ -4484,7 +4491,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -4528,7 +4535,7 @@
         <v>487</v>
       </c>
       <c r="U8" s="12" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="V8" s="3" t="s">
         <v>468</v>
@@ -4590,7 +4597,7 @@
         <v>494</v>
       </c>
       <c r="U9" s="12" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="V9" s="3" t="s">
         <v>468</v>
@@ -4602,13 +4609,13 @@
         <v>496</v>
       </c>
       <c r="Y9" s="12" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="Z9" s="4" t="s">
         <v>497</v>
       </c>
       <c r="AB9" s="4" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
     </row>
     <row r="10" spans="1:32" ht="409.5" x14ac:dyDescent="0.25">
@@ -4664,13 +4671,13 @@
         <v>496</v>
       </c>
       <c r="Y10" s="12" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="Z10" s="4" t="s">
         <v>497</v>
       </c>
       <c r="AB10" s="4" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="120" x14ac:dyDescent="0.25">
@@ -5157,7 +5164,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="135" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -5204,7 +5211,7 @@
         <v>501</v>
       </c>
       <c r="U19" s="12" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="V19" s="3" t="s">
         <v>468</v>
@@ -5263,7 +5270,7 @@
         <v>513</v>
       </c>
       <c r="U20" s="12" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="V20" s="3" t="s">
         <v>468</v>
@@ -5275,13 +5282,13 @@
         <v>482</v>
       </c>
       <c r="Y20" s="12" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="Z20" s="12" t="s">
         <v>514</v>
       </c>
       <c r="AB20" s="4" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
     </row>
     <row r="21" spans="1:28" ht="330" x14ac:dyDescent="0.25">
@@ -5310,7 +5317,7 @@
         <v>427</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="M21" s="4" t="s">
         <v>518</v>
@@ -5331,7 +5338,7 @@
         <v>521</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="V21" s="3" t="s">
         <v>468</v>
@@ -5343,13 +5350,13 @@
         <v>496</v>
       </c>
       <c r="Y21" s="12" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="Z21" s="4" t="s">
         <v>516</v>
       </c>
       <c r="AB21" s="4" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
     </row>
     <row r="22" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -5375,7 +5382,7 @@
         <v>353</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>517</v>
@@ -5396,7 +5403,7 @@
         <v>524</v>
       </c>
       <c r="U22" s="12" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="V22" s="3" t="s">
         <v>468</v>
@@ -5408,16 +5415,16 @@
         <v>496</v>
       </c>
       <c r="Y22" s="12" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="Z22" s="4" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="AB22" s="4" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28" ht="405" x14ac:dyDescent="0.25">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -5437,22 +5444,22 @@
         <v>347</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>511</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="U23" s="12" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="V23" s="3" t="s">
         <v>468</v>
@@ -5464,10 +5471,10 @@
         <v>482</v>
       </c>
       <c r="Y23" s="4" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="Z23" s="4" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
     </row>
     <row r="24" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -5514,7 +5521,7 @@
         <v>528</v>
       </c>
       <c r="U24" s="12" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="V24" s="3" t="s">
         <v>468</v>
@@ -5526,13 +5533,13 @@
         <v>496</v>
       </c>
       <c r="Y24" s="12" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="Z24" s="4" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="AB24" s="4" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="135" x14ac:dyDescent="0.25">
@@ -5588,10 +5595,10 @@
         <v>482</v>
       </c>
       <c r="Y25" s="12" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="AB25" s="4" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
     </row>
     <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -5661,7 +5668,7 @@
         <v>389</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>533</v>
@@ -5679,10 +5686,10 @@
         <v>520</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="U27" s="12" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="V27" s="3" t="s">
         <v>468</v>
@@ -5694,10 +5701,10 @@
         <v>496</v>
       </c>
       <c r="Y27" s="4" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="Z27" s="4" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
     </row>
     <row r="28" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -5723,7 +5730,7 @@
         <v>431</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="M28" s="4" t="s">
         <v>533</v>
@@ -5741,7 +5748,7 @@
         <v>520</v>
       </c>
       <c r="S28" s="4" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="V28" s="3" t="s">
         <v>468</v>
@@ -5756,7 +5763,7 @@
         <v>536</v>
       </c>
       <c r="Z28" s="4" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
     </row>
     <row r="29" spans="1:28" ht="135" x14ac:dyDescent="0.25">
@@ -5785,7 +5792,7 @@
         <v>389</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>537</v>
@@ -5803,10 +5810,10 @@
         <v>520</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="U29" s="12" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="V29" s="3" t="s">
         <v>468</v>
@@ -5818,10 +5825,10 @@
         <v>496</v>
       </c>
       <c r="Y29" s="4" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="Z29" s="4" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
     </row>
     <row r="30" spans="1:28" ht="75" x14ac:dyDescent="0.25">
@@ -5847,7 +5854,7 @@
         <v>431</v>
       </c>
       <c r="L30" s="4" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="M30" s="4" t="s">
         <v>537</v>
@@ -5865,7 +5872,7 @@
         <v>520</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="V30" s="3" t="s">
         <v>468</v>
@@ -5877,10 +5884,10 @@
         <v>496</v>
       </c>
       <c r="Y30" s="4" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="Z30" s="4" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -5965,7 +5972,7 @@
         <v>389</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="M32" s="4" t="s">
         <v>541</v>
@@ -6021,7 +6028,7 @@
         <v>431</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="M33" s="4" t="s">
         <v>541</v>
@@ -6074,7 +6081,7 @@
         <v>357</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="M34" s="4" t="s">
         <v>544</v>
@@ -6095,7 +6102,7 @@
         <v>547</v>
       </c>
       <c r="U34" s="12" t="s">
-        <v>880</v>
+        <v>873</v>
       </c>
       <c r="V34" s="3" t="s">
         <v>468</v>
@@ -6130,7 +6137,7 @@
         <v>347</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="M35" s="4" t="s">
         <v>544</v>
@@ -6163,7 +6170,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="330" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" ht="345" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -6210,7 +6217,7 @@
         <v>552</v>
       </c>
       <c r="U36" s="12" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="V36" s="3" t="s">
         <v>468</v>
@@ -6222,17 +6229,17 @@
         <v>554</v>
       </c>
       <c r="Y36" s="12" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="Z36" s="4" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="AA36" s="4"/>
       <c r="AB36" s="4" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="37" spans="1:28" ht="330" x14ac:dyDescent="0.25">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" ht="345" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -6279,7 +6286,7 @@
         <v>557</v>
       </c>
       <c r="U37" s="12" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="V37" s="3" t="s">
         <v>468</v>
@@ -6291,13 +6298,13 @@
         <v>554</v>
       </c>
       <c r="Y37" s="12" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="Z37" s="4" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="AB37" s="4" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
     </row>
     <row r="38" spans="1:28" ht="105" x14ac:dyDescent="0.25">
@@ -6326,7 +6333,7 @@
         <v>390</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="M38" s="4" t="s">
         <v>558</v>
@@ -6347,7 +6354,7 @@
         <v>560</v>
       </c>
       <c r="U38" s="12" t="s">
-        <v>881</v>
+        <v>874</v>
       </c>
       <c r="V38" s="3" t="s">
         <v>468</v>
@@ -6359,10 +6366,10 @@
         <v>496</v>
       </c>
       <c r="Y38" s="4" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="Z38" s="4" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
     </row>
     <row r="39" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -6429,7 +6436,7 @@
         <v>432</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="M40" s="4" t="s">
         <v>561</v>
@@ -6450,7 +6457,7 @@
         <v>565</v>
       </c>
       <c r="U40" s="12" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="V40" s="3" t="s">
         <v>468</v>
@@ -6462,7 +6469,7 @@
         <v>496</v>
       </c>
       <c r="Y40" s="4" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="Z40" s="4" t="s">
         <v>566</v>
@@ -6491,7 +6498,7 @@
         <v>361</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="M41" s="4" t="s">
         <v>567</v>
@@ -6527,7 +6534,7 @@
         <v>489</v>
       </c>
       <c r="AB41" s="4" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
     </row>
     <row r="42" spans="1:28" ht="90" x14ac:dyDescent="0.25">
@@ -6553,7 +6560,7 @@
         <v>362</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="M42" s="4" t="s">
         <v>572</v>
@@ -6586,13 +6593,13 @@
         <v>496</v>
       </c>
       <c r="Y42" s="12" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="Z42" s="4" t="s">
         <v>575</v>
       </c>
       <c r="AB42" s="4" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
     </row>
     <row r="43" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6618,7 +6625,7 @@
         <v>363</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="M43" s="4" t="s">
         <v>578</v>
@@ -6677,7 +6684,7 @@
         <v>363</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="M44" s="4" t="s">
         <v>579</v>
@@ -6751,7 +6758,7 @@
         <v>474</v>
       </c>
       <c r="Z45" s="4" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
     </row>
     <row r="46" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -6780,7 +6787,7 @@
         <v>392</v>
       </c>
       <c r="L46" s="4" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="M46" s="4" t="s">
         <v>583</v>
@@ -6792,7 +6799,7 @@
         <v>583</v>
       </c>
       <c r="P46" s="4" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="R46" s="3" t="s">
         <v>487</v>
@@ -6804,7 +6811,7 @@
         <v>363</v>
       </c>
       <c r="U46" s="12" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="V46" s="3" t="s">
         <v>468</v>
@@ -6819,7 +6826,7 @@
         <v>489</v>
       </c>
       <c r="Z46" s="4" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="47" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6845,7 +6852,7 @@
         <v>363</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="M47" s="4" t="s">
         <v>588</v>
@@ -7103,25 +7110,25 @@
         <v>366</v>
       </c>
       <c r="L53" s="4" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="M53" s="4" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="N53" s="4" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="O53" s="4" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="P53" s="4" t="s">
         <v>538</v>
       </c>
       <c r="S53" s="4" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="U53" s="12" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="V53" s="3" t="s">
         <v>468</v>
@@ -7133,13 +7140,13 @@
         <v>496</v>
       </c>
       <c r="Y53" s="4" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="Z53" s="4" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="AB53" s="4" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="54" spans="1:28" ht="225" x14ac:dyDescent="0.25">
@@ -7180,13 +7187,13 @@
         <v>593</v>
       </c>
       <c r="P54" s="4" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="S54" s="4" t="s">
         <v>594</v>
       </c>
       <c r="U54" s="12" t="s">
-        <v>833</v>
+        <v>883</v>
       </c>
       <c r="V54" s="3" t="s">
         <v>468</v>
@@ -7197,11 +7204,11 @@
       <c r="X54" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="Y54" s="4" t="s">
-        <v>782</v>
+      <c r="Y54" s="12" t="s">
+        <v>882</v>
       </c>
       <c r="Z54" s="12" t="s">
-        <v>834</v>
+        <v>828</v>
       </c>
     </row>
     <row r="55" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -7227,7 +7234,7 @@
         <v>434</v>
       </c>
       <c r="L55" s="4" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="M55" s="4" t="s">
         <v>598</v>
@@ -7251,13 +7258,13 @@
         <v>495</v>
       </c>
       <c r="X55" s="3" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="Y55" s="4" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="Z55" s="4" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
     </row>
     <row r="56" spans="1:28" ht="180" x14ac:dyDescent="0.25">
@@ -7286,7 +7293,7 @@
         <v>435</v>
       </c>
       <c r="L56" s="4" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="M56" s="4" t="s">
         <v>604</v>
@@ -7304,7 +7311,7 @@
         <v>607</v>
       </c>
       <c r="U56" s="12" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
       <c r="V56" s="3" t="s">
         <v>468</v>
@@ -7319,7 +7326,7 @@
         <v>608</v>
       </c>
       <c r="Z56" s="4" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
     </row>
     <row r="57" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -7345,7 +7352,7 @@
         <v>436</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="M57" s="4" t="s">
         <v>601</v>
@@ -7363,7 +7370,7 @@
         <v>609</v>
       </c>
       <c r="U57" s="12" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
       <c r="V57" s="3" t="s">
         <v>468</v>
@@ -7378,7 +7385,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="58" spans="1:28" ht="165" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:28" ht="255" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -7404,25 +7411,25 @@
         <v>398</v>
       </c>
       <c r="L58" s="4" t="s">
-        <v>610</v>
+        <v>877</v>
       </c>
       <c r="M58" s="4" t="s">
-        <v>611</v>
+        <v>878</v>
       </c>
       <c r="N58" s="3" t="s">
         <v>602</v>
       </c>
       <c r="O58" s="4" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="P58" s="4" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="S58" s="4" t="s">
-        <v>614</v>
+        <v>879</v>
       </c>
       <c r="U58" s="12" t="s">
-        <v>836</v>
+        <v>880</v>
       </c>
       <c r="V58" s="3" t="s">
         <v>468</v>
@@ -7433,11 +7440,11 @@
       <c r="X58" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="Y58" s="4" t="s">
-        <v>615</v>
+      <c r="Y58" s="12" t="s">
+        <v>881</v>
       </c>
       <c r="Z58" s="4" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
     </row>
     <row r="59" spans="1:28" ht="75" x14ac:dyDescent="0.25">
@@ -7463,22 +7470,22 @@
         <v>353</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="M59" s="4" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="O59" s="4" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="S59" s="4" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>837</v>
+        <v>830</v>
       </c>
       <c r="V59" s="3" t="s">
         <v>468</v>
@@ -7490,7 +7497,7 @@
         <v>496</v>
       </c>
       <c r="Y59" s="4" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
     </row>
     <row r="60" spans="1:28" ht="165" x14ac:dyDescent="0.25">
@@ -7519,19 +7526,19 @@
         <v>437</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="M60" s="4" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="N60" s="3" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="O60" s="4" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="S60" s="4" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="V60" s="3" t="s">
         <v>468</v>
@@ -7543,10 +7550,10 @@
         <v>496</v>
       </c>
       <c r="Y60" s="4" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="61" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="61" spans="1:28" ht="135" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -7569,22 +7576,22 @@
         <v>438</v>
       </c>
       <c r="L61" s="4" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="M61" s="4" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="O61" s="4" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="P61" s="4" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="S61" s="4" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="V61" s="3" t="s">
         <v>474</v>
@@ -7599,7 +7606,7 @@
         <v>474</v>
       </c>
       <c r="Z61" s="4" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
     </row>
     <row r="62" spans="1:28" ht="165" x14ac:dyDescent="0.25">
@@ -7628,25 +7635,25 @@
         <v>439</v>
       </c>
       <c r="L62" s="3" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="M62" s="4" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="N62" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O62" s="4" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="P62" s="4" t="s">
         <v>535</v>
       </c>
       <c r="S62" s="4" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="U62" s="12" t="s">
-        <v>838</v>
+        <v>831</v>
       </c>
       <c r="V62" s="3" t="s">
         <v>468</v>
@@ -7658,10 +7665,10 @@
         <v>482</v>
       </c>
       <c r="Y62" s="4" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="Z62" s="4" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
     </row>
     <row r="63" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -7763,25 +7770,25 @@
         <v>440</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="M65" s="4" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O65" s="4" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="P65" s="4" t="s">
         <v>535</v>
       </c>
       <c r="S65" s="4" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="U65" s="12" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
       <c r="V65" s="3" t="s">
         <v>468</v>
@@ -7796,7 +7803,7 @@
         <v>474</v>
       </c>
       <c r="Z65" s="4" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
     </row>
     <row r="66" spans="1:28" ht="165" x14ac:dyDescent="0.25">
@@ -7825,25 +7832,25 @@
         <v>439</v>
       </c>
       <c r="L66" s="3" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="M66" s="4" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="N66" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O66" s="4" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="P66" s="4" t="s">
         <v>535</v>
       </c>
       <c r="S66" s="4" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="U66" s="12" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
       <c r="V66" s="3" t="s">
         <v>474</v>
@@ -7899,7 +7906,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="68" spans="1:28" ht="210" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:28" ht="225" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -7907,7 +7914,7 @@
         <v>465</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>214</v>
@@ -7925,22 +7932,22 @@
         <v>399</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="M68" s="4" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="N68" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O68" s="4" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="P68" s="4" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="S68" s="4" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="U68" s="12"/>
       <c r="V68" s="5" t="s">
@@ -7953,16 +7960,16 @@
         <v>496</v>
       </c>
       <c r="Y68" s="12" t="s">
-        <v>842</v>
+        <v>835</v>
       </c>
       <c r="Z68" s="12" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="AB68" s="4" t="s">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="69" spans="1:28" ht="210" x14ac:dyDescent="0.25">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" ht="225" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -7985,25 +7992,25 @@
         <v>441</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="M69" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="N69" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="O69" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="P69" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="S69" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="T69" s="3" t="s">
         <v>636</v>
-      </c>
-      <c r="N69" s="3" t="s">
-        <v>627</v>
-      </c>
-      <c r="O69" s="4" t="s">
-        <v>637</v>
-      </c>
-      <c r="P69" s="4" t="s">
-        <v>638</v>
-      </c>
-      <c r="S69" s="4" t="s">
-        <v>639</v>
-      </c>
-      <c r="T69" s="3" t="s">
-        <v>640</v>
       </c>
       <c r="U69" s="12"/>
       <c r="V69" s="5" t="s">
@@ -8016,13 +8023,13 @@
         <v>496</v>
       </c>
       <c r="Y69" s="12" t="s">
-        <v>843</v>
+        <v>836</v>
       </c>
       <c r="Z69" s="12" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="AB69" s="4" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
     </row>
     <row r="70" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -8130,7 +8137,7 @@
         <v>472</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>882</v>
+        <v>875</v>
       </c>
       <c r="V72" s="3" t="s">
         <v>474</v>
@@ -8145,10 +8152,10 @@
         <v>474</v>
       </c>
       <c r="Z72" s="4" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="AB72" s="4" t="s">
-        <v>883</v>
+        <v>876</v>
       </c>
     </row>
     <row r="73" spans="1:28" ht="210" x14ac:dyDescent="0.25">
@@ -8177,25 +8184,25 @@
         <v>425</v>
       </c>
       <c r="L73" s="4" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="M73" s="4" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="N73" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O73" s="4" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="P73" s="4" t="s">
         <v>573</v>
       </c>
       <c r="S73" s="4" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>845</v>
+        <v>838</v>
       </c>
       <c r="V73" s="3" t="s">
         <v>468</v>
@@ -8207,13 +8214,13 @@
         <v>496</v>
       </c>
       <c r="Y73" s="4" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="Z73" s="4" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="AB73" s="4" t="s">
-        <v>844</v>
+        <v>837</v>
       </c>
     </row>
     <row r="74" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -8242,22 +8249,22 @@
         <v>425</v>
       </c>
       <c r="L74" s="4" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="M74" s="4" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="N74" s="3" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="O74" s="4" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="P74" s="4" t="s">
         <v>573</v>
       </c>
       <c r="S74" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V74" s="3" t="s">
         <v>468</v>
@@ -8269,10 +8276,10 @@
         <v>496</v>
       </c>
       <c r="Y74" s="4" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="Z74" s="4" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
     </row>
     <row r="75" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -8374,22 +8381,22 @@
         <v>444</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="M77" s="4" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="N77" s="3" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="O77" s="4" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="P77" s="4" t="s">
         <v>573</v>
       </c>
       <c r="S77" s="4" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="V77" s="3" t="s">
         <v>468</v>
@@ -8401,7 +8408,7 @@
         <v>482</v>
       </c>
       <c r="Y77" s="4" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
     </row>
     <row r="78" spans="1:28" ht="360" x14ac:dyDescent="0.25">
@@ -8430,28 +8437,28 @@
         <v>445</v>
       </c>
       <c r="L78" s="4" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="M78" s="4" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="N78" s="4" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="O78" s="4" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="P78" s="4" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="R78" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S78" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U78" s="12" t="s">
-        <v>846</v>
+        <v>839</v>
       </c>
       <c r="V78" s="3" t="s">
         <v>468</v>
@@ -8463,10 +8470,10 @@
         <v>496</v>
       </c>
       <c r="Y78" s="4" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="AB78" s="4" t="s">
-        <v>847</v>
+        <v>840</v>
       </c>
     </row>
     <row r="79" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8498,16 +8505,16 @@
         <v>445</v>
       </c>
       <c r="L79" s="3" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="M79" s="4" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="N79" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O79" s="4" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="P79" s="4" t="s">
         <v>531</v>
@@ -8516,10 +8523,10 @@
         <v>480</v>
       </c>
       <c r="S79" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U79" s="12" t="s">
-        <v>849</v>
+        <v>842</v>
       </c>
       <c r="V79" s="3" t="s">
         <v>468</v>
@@ -8531,10 +8538,10 @@
         <v>482</v>
       </c>
       <c r="Y79" s="12" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="AB79" s="4" t="s">
-        <v>848</v>
+        <v>841</v>
       </c>
     </row>
     <row r="80" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8566,16 +8573,16 @@
         <v>445</v>
       </c>
       <c r="L80" s="3" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="M80" s="4" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="N80" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O80" s="4" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="P80" s="4" t="s">
         <v>531</v>
@@ -8584,10 +8591,10 @@
         <v>480</v>
       </c>
       <c r="S80" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U80" s="12" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
       <c r="V80" s="3" t="s">
         <v>468</v>
@@ -8599,7 +8606,7 @@
         <v>482</v>
       </c>
       <c r="Y80" s="3" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="81" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8631,16 +8638,16 @@
         <v>445</v>
       </c>
       <c r="L81" s="3" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="M81" s="4" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="N81" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="O81" s="4" t="s">
         <v>657</v>
-      </c>
-      <c r="O81" s="4" t="s">
-        <v>661</v>
       </c>
       <c r="P81" s="4" t="s">
         <v>531</v>
@@ -8649,7 +8656,7 @@
         <v>480</v>
       </c>
       <c r="S81" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V81" s="3" t="s">
         <v>468</v>
@@ -8661,7 +8668,7 @@
         <v>482</v>
       </c>
       <c r="Y81" s="3" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="82" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8693,16 +8700,16 @@
         <v>445</v>
       </c>
       <c r="L82" s="3" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="M82" s="4" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="N82" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O82" s="4" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="P82" s="4" t="s">
         <v>531</v>
@@ -8711,7 +8718,7 @@
         <v>480</v>
       </c>
       <c r="S82" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V82" s="3" t="s">
         <v>468</v>
@@ -8723,7 +8730,7 @@
         <v>482</v>
       </c>
       <c r="Y82" s="3" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="83" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8755,16 +8762,16 @@
         <v>445</v>
       </c>
       <c r="L83" s="3" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="M83" s="4" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="N83" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O83" s="4" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="P83" s="4" t="s">
         <v>531</v>
@@ -8773,7 +8780,7 @@
         <v>480</v>
       </c>
       <c r="S83" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V83" s="3" t="s">
         <v>468</v>
@@ -8785,7 +8792,7 @@
         <v>482</v>
       </c>
       <c r="Y83" s="3" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="84" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8861,25 +8868,25 @@
         <v>445</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="M85" s="4" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="N85" s="3" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="O85" s="4" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="P85" s="4" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="R85" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S85" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V85" s="3" t="s">
         <v>468</v>
@@ -8891,7 +8898,7 @@
         <v>482</v>
       </c>
       <c r="Y85" s="3" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="86" spans="1:28" ht="240" x14ac:dyDescent="0.25">
@@ -8923,28 +8930,28 @@
         <v>445</v>
       </c>
       <c r="L86" s="4" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="M86" s="4" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="N86" s="3" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="P86" s="4" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="R86" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S86" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U86" s="12" t="s">
-        <v>851</v>
+        <v>844</v>
       </c>
       <c r="V86" s="3" t="s">
         <v>468</v>
@@ -8956,10 +8963,10 @@
         <v>496</v>
       </c>
       <c r="Y86" s="4" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="Z86" s="4" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
     </row>
     <row r="87" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -8991,16 +8998,16 @@
         <v>445</v>
       </c>
       <c r="L87" s="4" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="M87" s="4" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="N87" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O87" s="4" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="P87" s="4" t="s">
         <v>531</v>
@@ -9009,10 +9016,10 @@
         <v>480</v>
       </c>
       <c r="S87" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U87" s="12" t="s">
-        <v>852</v>
+        <v>845</v>
       </c>
       <c r="V87" s="3" t="s">
         <v>468</v>
@@ -9024,7 +9031,7 @@
         <v>482</v>
       </c>
       <c r="Y87" s="4" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
     </row>
     <row r="88" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -9056,16 +9063,16 @@
         <v>445</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="M88" s="4" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="N88" s="3" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="O88" s="4" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="P88" s="4" t="s">
         <v>569</v>
@@ -9074,7 +9081,7 @@
         <v>480</v>
       </c>
       <c r="S88" s="4" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="V88" s="3" t="s">
         <v>468</v>
@@ -9086,7 +9093,7 @@
         <v>482</v>
       </c>
       <c r="Y88" s="4" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
     </row>
     <row r="89" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -9153,16 +9160,16 @@
         <v>445</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="M90" s="4" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="N90" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O90" s="4" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="P90" s="4" t="s">
         <v>531</v>
@@ -9171,7 +9178,7 @@
         <v>480</v>
       </c>
       <c r="S90" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V90" s="3" t="s">
         <v>468</v>
@@ -9183,7 +9190,7 @@
         <v>482</v>
       </c>
       <c r="Y90" s="4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="91" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9212,25 +9219,25 @@
         <v>445</v>
       </c>
       <c r="L91" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M91" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N91" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O91" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P91" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R91" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S91" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V91" s="3" t="s">
         <v>468</v>
@@ -9242,13 +9249,13 @@
         <v>496</v>
       </c>
       <c r="Y91" s="12" t="s">
-        <v>854</v>
+        <v>847</v>
       </c>
       <c r="Z91" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB91" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="92" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9277,25 +9284,25 @@
         <v>445</v>
       </c>
       <c r="L92" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M92" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N92" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O92" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P92" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R92" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S92" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V92" s="3" t="s">
         <v>468</v>
@@ -9307,13 +9314,13 @@
         <v>496</v>
       </c>
       <c r="Y92" s="12" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
       <c r="Z92" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB92" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="93" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9342,25 +9349,25 @@
         <v>445</v>
       </c>
       <c r="L93" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M93" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N93" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O93" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P93" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R93" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S93" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V93" s="3" t="s">
         <v>468</v>
@@ -9372,13 +9379,13 @@
         <v>496</v>
       </c>
       <c r="Y93" s="12" t="s">
-        <v>856</v>
+        <v>849</v>
       </c>
       <c r="Z93" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB93" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="94" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9407,25 +9414,25 @@
         <v>445</v>
       </c>
       <c r="L94" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M94" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N94" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O94" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P94" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R94" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S94" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V94" s="3" t="s">
         <v>468</v>
@@ -9437,13 +9444,13 @@
         <v>496</v>
       </c>
       <c r="Y94" s="12" t="s">
-        <v>857</v>
+        <v>850</v>
       </c>
       <c r="Z94" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB94" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="95" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9472,25 +9479,25 @@
         <v>445</v>
       </c>
       <c r="L95" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M95" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N95" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O95" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P95" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R95" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S95" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V95" s="3" t="s">
         <v>468</v>
@@ -9502,13 +9509,13 @@
         <v>496</v>
       </c>
       <c r="Y95" s="12" t="s">
-        <v>858</v>
+        <v>851</v>
       </c>
       <c r="Z95" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB95" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="96" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9537,25 +9544,25 @@
         <v>445</v>
       </c>
       <c r="L96" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M96" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N96" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O96" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P96" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R96" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S96" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V96" s="3" t="s">
         <v>468</v>
@@ -9567,13 +9574,13 @@
         <v>496</v>
       </c>
       <c r="Y96" s="12" t="s">
-        <v>859</v>
+        <v>852</v>
       </c>
       <c r="Z96" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB96" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="97" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9602,25 +9609,25 @@
         <v>445</v>
       </c>
       <c r="L97" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M97" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N97" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O97" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P97" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R97" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S97" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V97" s="3" t="s">
         <v>468</v>
@@ -9632,13 +9639,13 @@
         <v>496</v>
       </c>
       <c r="Y97" s="12" t="s">
-        <v>860</v>
+        <v>853</v>
       </c>
       <c r="Z97" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB97" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="98" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9667,25 +9674,25 @@
         <v>445</v>
       </c>
       <c r="L98" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M98" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N98" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O98" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P98" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R98" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S98" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V98" s="3" t="s">
         <v>468</v>
@@ -9697,13 +9704,13 @@
         <v>496</v>
       </c>
       <c r="Y98" s="12" t="s">
-        <v>861</v>
+        <v>854</v>
       </c>
       <c r="Z98" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB98" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="99" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9732,25 +9739,25 @@
         <v>445</v>
       </c>
       <c r="L99" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M99" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N99" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O99" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P99" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R99" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S99" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V99" s="3" t="s">
         <v>468</v>
@@ -9762,13 +9769,13 @@
         <v>496</v>
       </c>
       <c r="Y99" s="12" t="s">
-        <v>863</v>
+        <v>856</v>
       </c>
       <c r="Z99" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB99" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="100" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9797,25 +9804,25 @@
         <v>445</v>
       </c>
       <c r="L100" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M100" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N100" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O100" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P100" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R100" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S100" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V100" s="3" t="s">
         <v>468</v>
@@ -9827,13 +9834,13 @@
         <v>496</v>
       </c>
       <c r="Y100" s="12" t="s">
-        <v>862</v>
+        <v>855</v>
       </c>
       <c r="Z100" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB100" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="101" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9862,25 +9869,25 @@
         <v>445</v>
       </c>
       <c r="L101" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M101" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N101" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O101" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P101" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R101" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S101" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V101" s="3" t="s">
         <v>468</v>
@@ -9892,13 +9899,13 @@
         <v>496</v>
       </c>
       <c r="Y101" s="12" t="s">
-        <v>864</v>
+        <v>857</v>
       </c>
       <c r="Z101" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB101" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="102" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9927,25 +9934,25 @@
         <v>445</v>
       </c>
       <c r="L102" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M102" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N102" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O102" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P102" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R102" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S102" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V102" s="3" t="s">
         <v>468</v>
@@ -9957,13 +9964,13 @@
         <v>496</v>
       </c>
       <c r="Y102" s="12" t="s">
-        <v>865</v>
+        <v>858</v>
       </c>
       <c r="Z102" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB102" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="103" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -9992,25 +9999,25 @@
         <v>445</v>
       </c>
       <c r="L103" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M103" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N103" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O103" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P103" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R103" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S103" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V103" s="3" t="s">
         <v>468</v>
@@ -10022,13 +10029,13 @@
         <v>496</v>
       </c>
       <c r="Y103" s="12" t="s">
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="Z103" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB103" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="104" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10057,25 +10064,25 @@
         <v>445</v>
       </c>
       <c r="L104" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M104" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N104" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O104" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P104" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R104" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S104" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V104" s="3" t="s">
         <v>468</v>
@@ -10087,13 +10094,13 @@
         <v>496</v>
       </c>
       <c r="Y104" s="12" t="s">
-        <v>867</v>
+        <v>860</v>
       </c>
       <c r="Z104" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB104" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="105" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10122,25 +10129,25 @@
         <v>445</v>
       </c>
       <c r="L105" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M105" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N105" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O105" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P105" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R105" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S105" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V105" s="3" t="s">
         <v>468</v>
@@ -10152,13 +10159,13 @@
         <v>496</v>
       </c>
       <c r="Y105" s="12" t="s">
-        <v>868</v>
+        <v>861</v>
       </c>
       <c r="Z105" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB105" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="106" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10187,25 +10194,25 @@
         <v>445</v>
       </c>
       <c r="L106" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M106" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N106" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O106" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P106" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R106" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S106" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V106" s="3" t="s">
         <v>468</v>
@@ -10217,13 +10224,13 @@
         <v>496</v>
       </c>
       <c r="Y106" s="12" t="s">
-        <v>869</v>
+        <v>862</v>
       </c>
       <c r="Z106" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB106" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="107" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10252,25 +10259,25 @@
         <v>445</v>
       </c>
       <c r="L107" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M107" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N107" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O107" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P107" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R107" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S107" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V107" s="3" t="s">
         <v>468</v>
@@ -10282,13 +10289,13 @@
         <v>496</v>
       </c>
       <c r="Y107" s="12" t="s">
-        <v>870</v>
+        <v>863</v>
       </c>
       <c r="Z107" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB107" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="108" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10317,25 +10324,25 @@
         <v>445</v>
       </c>
       <c r="L108" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M108" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N108" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O108" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P108" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R108" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S108" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V108" s="3" t="s">
         <v>468</v>
@@ -10347,13 +10354,13 @@
         <v>496</v>
       </c>
       <c r="Y108" s="12" t="s">
-        <v>871</v>
+        <v>864</v>
       </c>
       <c r="Z108" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB108" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="109" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
@@ -10382,25 +10389,25 @@
         <v>445</v>
       </c>
       <c r="L109" s="4" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="M109" s="4" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="N109" s="3" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="O109" s="4" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="P109" s="4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R109" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S109" s="4" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="V109" s="3" t="s">
         <v>468</v>
@@ -10412,13 +10419,13 @@
         <v>496</v>
       </c>
       <c r="Y109" s="12" t="s">
-        <v>872</v>
+        <v>865</v>
       </c>
       <c r="Z109" s="4" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="AB109" s="4" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
     </row>
     <row r="110" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10447,16 +10454,16 @@
         <v>445</v>
       </c>
       <c r="L110" s="3" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="M110" s="4" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="N110" s="3" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="O110" s="4" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="P110" s="4" t="s">
         <v>531</v>
@@ -10465,7 +10472,7 @@
         <v>480</v>
       </c>
       <c r="S110" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V110" s="3" t="s">
         <v>468</v>
@@ -10477,7 +10484,7 @@
         <v>482</v>
       </c>
       <c r="Y110" s="4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="111" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10588,22 +10595,22 @@
         <v>445</v>
       </c>
       <c r="L113" s="12" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="M113" s="12" t="s">
-        <v>877</v>
+        <v>870</v>
       </c>
       <c r="N113" s="3" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="O113" s="4" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="S113" s="12" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
       <c r="U113" s="12" t="s">
-        <v>873</v>
+        <v>866</v>
       </c>
       <c r="V113" s="3" t="s">
         <v>468</v>
@@ -10615,13 +10622,13 @@
         <v>496</v>
       </c>
       <c r="Y113" s="12" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="Z113" s="4" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="AB113" s="4" t="s">
-        <v>876</v>
+        <v>869</v>
       </c>
     </row>
     <row r="114" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10650,28 +10657,28 @@
         <v>445</v>
       </c>
       <c r="L114" s="4" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="M114" s="4" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="N114" s="3" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="O114" s="4" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="P114" s="4" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="R114" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S114" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="U114" s="12" t="s">
-        <v>879</v>
+        <v>872</v>
       </c>
       <c r="V114" s="3" t="s">
         <v>468</v>
@@ -10683,10 +10690,10 @@
         <v>496</v>
       </c>
       <c r="Y114" s="4" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="Z114" s="4" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
     </row>
     <row r="115" spans="1:28" ht="255" x14ac:dyDescent="0.25">
@@ -10715,25 +10722,25 @@
         <v>445</v>
       </c>
       <c r="L115" s="4" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="M115" s="4" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="N115" s="3" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="O115" s="4" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="P115" s="4" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="R115" s="3" t="s">
         <v>480</v>
       </c>
       <c r="S115" s="4" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="V115" s="3" t="s">
         <v>468</v>
@@ -10745,10 +10752,10 @@
         <v>496</v>
       </c>
       <c r="Y115" s="4" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="Z115" s="4" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
     </row>
     <row r="116" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -10926,22 +10933,22 @@
         <v>408</v>
       </c>
       <c r="L120" s="4" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="M120" s="4" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="N120" s="3" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="O120" s="4" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="P120" s="4" t="s">
         <v>595</v>
       </c>
       <c r="S120" s="4" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="V120" s="3" t="s">
         <v>468</v>
@@ -10953,10 +10960,10 @@
         <v>496</v>
       </c>
       <c r="Y120" s="4" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="Z120" s="4" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
     </row>
     <row r="121" spans="1:28" ht="30" x14ac:dyDescent="0.25">

</xml_diff>